<commit_message>
refactor: stabilize cockpit, mandate UTF-8 globally to fix mojibake, add in-memory unit tests, and perform git cleanup
</commit_message>
<xml_diff>
--- a/ro_workstation/data/mis/archive/20240331.xlsx
+++ b/ro_workstation/data/mis/archive/20240331.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>S No</t>
   </si>
@@ -103,6 +103,33 @@
   </si>
   <si>
     <t>ADV</t>
+  </si>
+  <si>
+    <t>Cash on Hand</t>
+  </si>
+  <si>
+    <t>ATM Cash</t>
+  </si>
+  <si>
+    <t>BC Cash</t>
+  </si>
+  <si>
+    <t>BNA Cash</t>
+  </si>
+  <si>
+    <t>Total Cash</t>
+  </si>
+  <si>
+    <t>CRL</t>
+  </si>
+  <si>
+    <t>Excess</t>
+  </si>
+  <si>
+    <t>Bulk Dep</t>
+  </si>
+  <si>
+    <t>PL</t>
   </si>
 </sst>
 </file>
@@ -592,10 +619,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89E97327-3999-4161-AA71-04A7E08FE8D2}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:AW56"/>
+  <dimension ref="A1:AI56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:26" ht="15">
+    <row r="1" spans="1:35" ht="15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -674,8 +701,35 @@
       <c r="Z1" s="3" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:49" ht="15">
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" ht="15">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -763,20 +817,6 @@
       <c r="AG2" s="6"/>
       <c r="AH2" s="6"/>
       <c r="AI2" s="6"/>
-      <c r="AJ2" s="6"/>
-      <c r="AK2" s="6"/>
-      <c r="AL2" s="6"/>
-      <c r="AM2" s="6"/>
-      <c r="AN2" s="6"/>
-      <c r="AO2" s="6"/>
-      <c r="AP2" s="6"/>
-      <c r="AQ2" s="6"/>
-      <c r="AR2" s="6"/>
-      <c r="AS2" s="6"/>
-      <c r="AT2" s="6"/>
-      <c r="AU2" s="6"/>
-      <c r="AV2" s="6"/>
-      <c r="AW2" s="6"/>
     </row>
     <row r="3" spans="1:26" ht="15">
       <c r="A3" s="1">

</xml_diff>